<commit_message>
TemplateMap.xlsx example variable name change
</commit_message>
<xml_diff>
--- a/Autogen/TemplateMap.xlsx
+++ b/Autogen/TemplateMap.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29404"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF53B3EC-5234-4185-8C5B-B65F66B19071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E91953FF-73EF-4D8F-BBDD-165AB26952C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
     <t>Widget</t>
   </si>
   <si>
-    <t>Example</t>
+    <t>Example Var</t>
   </si>
   <si>
     <t>uint8_t</t>
@@ -911,7 +911,7 @@
     <col min="10" max="10" width="13.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="24" customHeight="1">
+    <row r="1" spans="1:10" ht="39" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Autogen NVM storage fix + bus update active node ptr handling changes
</commit_message>
<xml_diff>
--- a/Autogen/TemplateMap.xlsx
+++ b/Autogen/TemplateMap.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29404"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E91953FF-73EF-4D8F-BBDD-165AB26952C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CAB1073E-F18A-4EAF-909D-2AF167EF6289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -66,7 +66,7 @@
     <t>Widget</t>
   </si>
   <si>
-    <t>Example Var</t>
+    <t>Example</t>
   </si>
   <si>
     <t>uint8_t</t>

</xml_diff>

<commit_message>
Initial untested auto-migration implementation and Hub/Node VarInfo_t separation.
</commit_message>
<xml_diff>
--- a/Autogen/TemplateMap.xlsx
+++ b/Autogen/TemplateMap.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30305"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CAB1073E-F18A-4EAF-909D-2AF167EF6289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{33F61A04-EA72-484C-86C5-D1F423725CBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
-    <t>Var ID</t>
+    <t>Var Name</t>
   </si>
   <si>
     <t>Data Type</t>
@@ -127,7 +127,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -246,56 +246,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -307,24 +262,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -339,6 +276,15 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -579,7 +525,7 @@
     </dxf>
     <dxf>
       <border>
-        <bottom style="medium">
+        <bottom style="thin">
           <color rgb="FF000000"/>
         </bottom>
       </border>
@@ -706,7 +652,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Table11011" displayName="Table11011" ref="A1:J42" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowBorderDxfId="11" tableBorderDxfId="12" totalsRowBorderDxfId="10">
   <autoFilter ref="A1:J42" xr:uid="{00000000-0009-0000-0100-000003000000}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Var ID" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Var Name" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Data Type" dataDxfId="8"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="External Access" dataDxfId="7"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Units" dataDxfId="6"/>
@@ -717,7 +663,7 @@
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0200-000009000000}" name="Description" dataDxfId="1"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0200-00000A000000}" name="Widget" dataDxfId="0"/>
   </tableColumns>
-  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -912,71 +858,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="39" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="J1" s="11" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="E2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="8" t="s">
+      <c r="G2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="8" t="s">
+      <c r="I2" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="9"/>
+      <c r="A3" s="6"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
@@ -985,10 +931,10 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="I3" s="3"/>
-      <c r="J3" s="11"/>
+      <c r="J3" s="5"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="12"/>
+      <c r="A4" s="6"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
@@ -997,10 +943,10 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
-      <c r="J4" s="11"/>
+      <c r="J4" s="5"/>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="12"/>
+      <c r="A5" s="6"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="D5" s="3"/>
@@ -1009,10 +955,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
-      <c r="J5" s="11"/>
+      <c r="J5" s="5"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="12"/>
+      <c r="A6" s="6"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -1021,10 +967,10 @@
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
-      <c r="J6" s="11"/>
+      <c r="J6" s="5"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="12"/>
+      <c r="A7" s="6"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
       <c r="D7" s="3"/>
@@ -1033,10 +979,10 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
-      <c r="J7" s="11"/>
+      <c r="J7" s="5"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="12"/>
+      <c r="A8" s="6"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
       <c r="D8" s="3"/>
@@ -1045,10 +991,10 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
-      <c r="J8" s="11"/>
+      <c r="J8" s="5"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="12"/>
+      <c r="A9" s="6"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
       <c r="D9" s="3"/>
@@ -1057,10 +1003,10 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
-      <c r="J9" s="11"/>
+      <c r="J9" s="5"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="12"/>
+      <c r="A10" s="6"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
       <c r="D10" s="3"/>
@@ -1069,10 +1015,10 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
-      <c r="J10" s="11"/>
+      <c r="J10" s="5"/>
     </row>
     <row r="11" spans="1:10">
-      <c r="A11" s="12"/>
+      <c r="A11" s="6"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
       <c r="D11" s="3"/>
@@ -1081,10 +1027,10 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
-      <c r="J11" s="11"/>
+      <c r="J11" s="5"/>
     </row>
     <row r="12" spans="1:10" ht="15" customHeight="1">
-      <c r="A12" s="12"/>
+      <c r="A12" s="6"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
       <c r="D12" s="3"/>
@@ -1093,10 +1039,10 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="I12" s="3"/>
-      <c r="J12" s="11"/>
+      <c r="J12" s="5"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="12"/>
+      <c r="A13" s="6"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
@@ -1105,10 +1051,10 @@
       <c r="G13" s="3"/>
       <c r="H13" s="3"/>
       <c r="I13" s="3"/>
-      <c r="J13" s="11"/>
+      <c r="J13" s="5"/>
     </row>
     <row r="14" spans="1:10" ht="15" customHeight="1">
-      <c r="A14" s="12"/>
+      <c r="A14" s="6"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
@@ -1117,10 +1063,10 @@
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
-      <c r="J14" s="11"/>
+      <c r="J14" s="5"/>
     </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="12"/>
+      <c r="A15" s="6"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
@@ -1129,10 +1075,10 @@
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
-      <c r="J15" s="11"/>
+      <c r="J15" s="5"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="12"/>
+      <c r="A16" s="6"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
       <c r="D16" s="3"/>
@@ -1141,10 +1087,10 @@
       <c r="G16" s="3"/>
       <c r="H16" s="3"/>
       <c r="I16" s="3"/>
-      <c r="J16" s="11"/>
+      <c r="J16" s="5"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="12"/>
+      <c r="A17" s="6"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
       <c r="D17" s="3"/>
@@ -1153,10 +1099,10 @@
       <c r="G17" s="3"/>
       <c r="H17" s="3"/>
       <c r="I17" s="3"/>
-      <c r="J17" s="11"/>
+      <c r="J17" s="5"/>
     </row>
     <row r="18" spans="1:10">
-      <c r="A18" s="12"/>
+      <c r="A18" s="6"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
       <c r="D18" s="3"/>
@@ -1165,10 +1111,10 @@
       <c r="G18" s="3"/>
       <c r="H18" s="3"/>
       <c r="I18" s="3"/>
-      <c r="J18" s="11"/>
+      <c r="J18" s="5"/>
     </row>
     <row r="19" spans="1:10">
-      <c r="A19" s="12"/>
+      <c r="A19" s="6"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
       <c r="D19" s="3"/>
@@ -1177,10 +1123,10 @@
       <c r="G19" s="3"/>
       <c r="H19" s="3"/>
       <c r="I19" s="3"/>
-      <c r="J19" s="11"/>
+      <c r="J19" s="5"/>
     </row>
     <row r="20" spans="1:10">
-      <c r="A20" s="12"/>
+      <c r="A20" s="6"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
@@ -1189,10 +1135,10 @@
       <c r="G20" s="3"/>
       <c r="H20" s="3"/>
       <c r="I20" s="3"/>
-      <c r="J20" s="11"/>
+      <c r="J20" s="5"/>
     </row>
     <row r="21" spans="1:10">
-      <c r="A21" s="12"/>
+      <c r="A21" s="6"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
@@ -1201,10 +1147,10 @@
       <c r="G21" s="3"/>
       <c r="H21" s="3"/>
       <c r="I21" s="3"/>
-      <c r="J21" s="11"/>
+      <c r="J21" s="5"/>
     </row>
     <row r="22" spans="1:10">
-      <c r="A22" s="12"/>
+      <c r="A22" s="6"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
       <c r="D22" s="3"/>
@@ -1213,10 +1159,10 @@
       <c r="G22" s="3"/>
       <c r="H22" s="3"/>
       <c r="I22" s="3"/>
-      <c r="J22" s="11"/>
+      <c r="J22" s="5"/>
     </row>
     <row r="23" spans="1:10">
-      <c r="A23" s="12"/>
+      <c r="A23" s="6"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
@@ -1225,10 +1171,10 @@
       <c r="G23" s="3"/>
       <c r="H23" s="3"/>
       <c r="I23" s="3"/>
-      <c r="J23" s="11"/>
+      <c r="J23" s="5"/>
     </row>
     <row r="24" spans="1:10">
-      <c r="A24" s="12"/>
+      <c r="A24" s="6"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
       <c r="D24" s="3"/>
@@ -1237,10 +1183,10 @@
       <c r="G24" s="3"/>
       <c r="H24" s="3"/>
       <c r="I24" s="3"/>
-      <c r="J24" s="11"/>
+      <c r="J24" s="5"/>
     </row>
     <row r="25" spans="1:10">
-      <c r="A25" s="12"/>
+      <c r="A25" s="6"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
@@ -1249,10 +1195,10 @@
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
       <c r="I25" s="3"/>
-      <c r="J25" s="11"/>
+      <c r="J25" s="5"/>
     </row>
     <row r="26" spans="1:10">
-      <c r="A26" s="12"/>
+      <c r="A26" s="6"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
@@ -1261,10 +1207,10 @@
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
       <c r="I26" s="3"/>
-      <c r="J26" s="11"/>
+      <c r="J26" s="5"/>
     </row>
     <row r="27" spans="1:10">
-      <c r="A27" s="12"/>
+      <c r="A27" s="6"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
       <c r="D27" s="3"/>
@@ -1273,10 +1219,10 @@
       <c r="G27" s="3"/>
       <c r="H27" s="3"/>
       <c r="I27" s="3"/>
-      <c r="J27" s="11"/>
+      <c r="J27" s="5"/>
     </row>
     <row r="28" spans="1:10">
-      <c r="A28" s="12"/>
+      <c r="A28" s="6"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
       <c r="D28" s="3"/>
@@ -1285,10 +1231,10 @@
       <c r="G28" s="3"/>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
-      <c r="J28" s="11"/>
+      <c r="J28" s="5"/>
     </row>
     <row r="29" spans="1:10">
-      <c r="A29" s="12"/>
+      <c r="A29" s="6"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
       <c r="D29" s="3"/>
@@ -1297,10 +1243,10 @@
       <c r="G29" s="3"/>
       <c r="H29" s="3"/>
       <c r="I29" s="3"/>
-      <c r="J29" s="11"/>
+      <c r="J29" s="5"/>
     </row>
     <row r="30" spans="1:10">
-      <c r="A30" s="12"/>
+      <c r="A30" s="6"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
       <c r="D30" s="3"/>
@@ -1309,10 +1255,10 @@
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
       <c r="I30" s="3"/>
-      <c r="J30" s="11"/>
+      <c r="J30" s="5"/>
     </row>
     <row r="31" spans="1:10">
-      <c r="A31" s="12"/>
+      <c r="A31" s="6"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
       <c r="D31" s="3"/>
@@ -1321,10 +1267,10 @@
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
       <c r="I31" s="3"/>
-      <c r="J31" s="11"/>
+      <c r="J31" s="5"/>
     </row>
     <row r="32" spans="1:10">
-      <c r="A32" s="12"/>
+      <c r="A32" s="6"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
       <c r="D32" s="3"/>
@@ -1333,10 +1279,10 @@
       <c r="G32" s="3"/>
       <c r="H32" s="3"/>
       <c r="I32" s="3"/>
-      <c r="J32" s="11"/>
+      <c r="J32" s="5"/>
     </row>
     <row r="33" spans="1:10">
-      <c r="A33" s="12"/>
+      <c r="A33" s="6"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
       <c r="D33" s="3"/>
@@ -1345,10 +1291,10 @@
       <c r="G33" s="3"/>
       <c r="H33" s="3"/>
       <c r="I33" s="3"/>
-      <c r="J33" s="11"/>
+      <c r="J33" s="5"/>
     </row>
     <row r="34" spans="1:10">
-      <c r="A34" s="12"/>
+      <c r="A34" s="6"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
       <c r="D34" s="3"/>
@@ -1357,10 +1303,10 @@
       <c r="G34" s="3"/>
       <c r="H34" s="3"/>
       <c r="I34" s="3"/>
-      <c r="J34" s="11"/>
+      <c r="J34" s="5"/>
     </row>
     <row r="35" spans="1:10">
-      <c r="A35" s="12"/>
+      <c r="A35" s="6"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
       <c r="D35" s="3"/>
@@ -1369,10 +1315,10 @@
       <c r="G35" s="3"/>
       <c r="H35" s="3"/>
       <c r="I35" s="3"/>
-      <c r="J35" s="11"/>
+      <c r="J35" s="5"/>
     </row>
     <row r="36" spans="1:10">
-      <c r="A36" s="12"/>
+      <c r="A36" s="6"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
       <c r="D36" s="3"/>
@@ -1381,10 +1327,10 @@
       <c r="G36" s="3"/>
       <c r="H36" s="3"/>
       <c r="I36" s="3"/>
-      <c r="J36" s="11"/>
+      <c r="J36" s="5"/>
     </row>
     <row r="37" spans="1:10">
-      <c r="A37" s="12"/>
+      <c r="A37" s="6"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
       <c r="D37" s="3"/>
@@ -1393,10 +1339,10 @@
       <c r="G37" s="3"/>
       <c r="H37" s="3"/>
       <c r="I37" s="3"/>
-      <c r="J37" s="11"/>
+      <c r="J37" s="5"/>
     </row>
     <row r="38" spans="1:10">
-      <c r="A38" s="12"/>
+      <c r="A38" s="6"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
       <c r="D38" s="3"/>
@@ -1405,10 +1351,10 @@
       <c r="G38" s="3"/>
       <c r="H38" s="3"/>
       <c r="I38" s="3"/>
-      <c r="J38" s="11"/>
+      <c r="J38" s="5"/>
     </row>
     <row r="39" spans="1:10">
-      <c r="A39" s="12"/>
+      <c r="A39" s="6"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
@@ -1417,10 +1363,10 @@
       <c r="G39" s="3"/>
       <c r="H39" s="3"/>
       <c r="I39" s="3"/>
-      <c r="J39" s="11"/>
+      <c r="J39" s="5"/>
     </row>
     <row r="40" spans="1:10">
-      <c r="A40" s="12"/>
+      <c r="A40" s="6"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
       <c r="D40" s="3"/>
@@ -1429,10 +1375,10 @@
       <c r="G40" s="3"/>
       <c r="H40" s="3"/>
       <c r="I40" s="3"/>
-      <c r="J40" s="11"/>
+      <c r="J40" s="5"/>
     </row>
     <row r="41" spans="1:10">
-      <c r="A41" s="12"/>
+      <c r="A41" s="6"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
       <c r="D41" s="3"/>
@@ -1441,10 +1387,10 @@
       <c r="G41" s="3"/>
       <c r="H41" s="3"/>
       <c r="I41" s="3"/>
-      <c r="J41" s="11"/>
+      <c r="J41" s="5"/>
     </row>
     <row r="42" spans="1:10">
-      <c r="A42" s="13"/>
+      <c r="A42" s="7"/>
       <c r="B42" s="4"/>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
@@ -1453,7 +1399,7 @@
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4"/>
-      <c r="J42" s="14"/>
+      <c r="J42" s="8"/>
     </row>
     <row r="43" spans="1:10">
       <c r="A43" s="2"/>

</xml_diff>